<commit_message>
Nuevo registro: Luz Mercedes
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4262,6 +4262,60 @@
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>124930.0</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TIENDA MAGDALENA AV. JOSE GALVEZ N°695</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>MILAGROS URBANO</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Monica Maria Damian De Los Rios</t>
+        </is>
+      </c>
+      <c r="F73" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>KÁBALA</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Luz Mercedes</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>20261007-01</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>